<commit_message>
Barcode Manuals Uploaded; Parts Selection
</commit_message>
<xml_diff>
--- a/Documents/Dev-Files/Component-Selection.xlsx
+++ b/Documents/Dev-Files/Component-Selection.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\AdamLucks-GateSecuritySystem\Documents\Dev-Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D91FA0BD-DE56-4540-8934-4E13A909F150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1493A5D0-B035-4A75-9565-F545DA870DDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Components" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
   <si>
     <t>S.No</t>
   </si>
@@ -75,9 +75,6 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>It is better if one is shipped to Pakistan for faster testing</t>
-  </si>
-  <si>
     <t>Any printer can be used provided it has a USB or an ethernet or WiFi interface</t>
   </si>
   <si>
@@ -94,6 +91,27 @@
   </si>
   <si>
     <t>UCTRONICS</t>
+  </si>
+  <si>
+    <t>Local Link</t>
+  </si>
+  <si>
+    <t>w11stop</t>
+  </si>
+  <si>
+    <t>circuit</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>4GB version will be used and ordered by Huzaifa</t>
+  </si>
+  <si>
+    <t>Will be ordered by Huzaifa</t>
+  </si>
+  <si>
+    <t>Will be ordered by Sir Hassan internationally. Link provided</t>
   </si>
 </sst>
 </file>
@@ -249,7 +267,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -288,12 +306,219 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="12">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -320,190 +545,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -518,15 +559,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{015DB811-CAAB-4CD9-A1D4-1C92075F62AD}" name="Table1" displayName="Table1" ref="A1:G6" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="2" tableBorderDxfId="3" totalsRowBorderDxfId="1">
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{18F54C0B-A7E8-4071-9EBF-DB3126C9CDE9}" name="S.No" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{317E679B-3A79-40C4-9272-4E4E6E311408}" name="Component Name" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{9AE403A4-D115-4AA5-9AE9-A19D297F28EB}" name="Description" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{CF1C59C6-6EE5-49E0-9094-40F8CE5E87A8}" name="Quantity" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{0DEF5A6D-DB44-4743-864E-972C7CD936F7}" name="Cost" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{A04DEE05-1D8F-43F3-A2DF-1BF2819B85CD}" name="Reference Link" dataDxfId="5" dataCellStyle="Hyperlink"/>
-    <tableColumn id="7" xr3:uid="{46EC11C6-2EAF-4885-9B5D-F5A79DA3565B}" name="Remarks" dataDxfId="4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{015DB811-CAAB-4CD9-A1D4-1C92075F62AD}" name="Table1" displayName="Table1" ref="A1:H6" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{18F54C0B-A7E8-4071-9EBF-DB3126C9CDE9}" name="S.No" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{317E679B-3A79-40C4-9272-4E4E6E311408}" name="Component Name" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{9AE403A4-D115-4AA5-9AE9-A19D297F28EB}" name="Description" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{CF1C59C6-6EE5-49E0-9094-40F8CE5E87A8}" name="Quantity" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{0DEF5A6D-DB44-4743-864E-972C7CD936F7}" name="Cost" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{A04DEE05-1D8F-43F3-A2DF-1BF2819B85CD}" name="Reference Link" dataDxfId="2" dataCellStyle="Hyperlink"/>
+    <tableColumn id="8" xr3:uid="{564315F0-111A-448F-8B4B-0DEE1B8A0A94}" name="Local Link" dataDxfId="0" dataCellStyle="Hyperlink"/>
+    <tableColumn id="7" xr3:uid="{46EC11C6-2EAF-4885-9B5D-F5A79DA3565B}" name="Remarks" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -795,19 +837,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.77734375" customWidth="1"/>
+    <col min="1" max="1" width="5.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="45.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.109375" customWidth="1"/>
     <col min="5" max="5" width="8.33203125" customWidth="1"/>
-    <col min="6" max="6" width="14.88671875" customWidth="1"/>
-    <col min="7" max="7" width="65" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="14.88671875" customWidth="1"/>
+    <col min="8" max="8" width="65" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -827,10 +869,13 @@
         <v>5</v>
       </c>
       <c r="G1" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="17" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -849,11 +894,14 @@
       <c r="F2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G2" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -872,19 +920,22 @@
       <c r="F3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G3" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>19</v>
       </c>
       <c r="D4" s="5">
         <v>1</v>
@@ -895,19 +946,22 @@
       <c r="F4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G4" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>21</v>
       </c>
       <c r="D5" s="5">
         <v>1</v>
@@ -916,13 +970,16 @@
         <v>27.99</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -941,124 +998,150 @@
       <c r="F6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="13" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G6" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D7" s="1"/>
       <c r="E7" s="2"/>
       <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D8" s="1"/>
       <c r="E8" s="2"/>
       <c r="F8" s="1"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D9" s="1"/>
       <c r="E9" s="2"/>
       <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D10" s="1"/>
       <c r="E10" s="2"/>
       <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D11" s="1"/>
       <c r="E11" s="2"/>
       <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D12" s="1"/>
       <c r="E12" s="2"/>
       <c r="F12" s="1"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D13" s="1"/>
       <c r="E13" s="2"/>
       <c r="F13" s="1"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D14" s="1"/>
       <c r="E14" s="2"/>
       <c r="F14" s="1"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D15" s="1"/>
       <c r="E15" s="2"/>
       <c r="F15" s="1"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D16" s="1"/>
       <c r="E16" s="2"/>
       <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="G16" s="1"/>
+    </row>
+    <row r="17" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D17" s="1"/>
       <c r="E17" s="2"/>
       <c r="F17" s="1"/>
-    </row>
-    <row r="18" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D18" s="1"/>
       <c r="E18" s="2"/>
       <c r="F18" s="1"/>
-    </row>
-    <row r="19" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="G18" s="1"/>
+    </row>
+    <row r="19" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D19" s="1"/>
       <c r="E19" s="2"/>
       <c r="F19" s="1"/>
-    </row>
-    <row r="20" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="G19" s="1"/>
+    </row>
+    <row r="20" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D20" s="1"/>
       <c r="E20" s="2"/>
       <c r="F20" s="1"/>
-    </row>
-    <row r="21" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="G20" s="1"/>
+    </row>
+    <row r="21" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="G21" s="1"/>
+    </row>
+    <row r="22" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
-    </row>
-    <row r="23" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="G22" s="1"/>
+    </row>
+    <row r="23" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
-    </row>
-    <row r="24" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="G23" s="1"/>
+    </row>
+    <row r="24" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
-    </row>
-    <row r="25" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="G24" s="1"/>
+    </row>
+    <row r="25" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
-    </row>
-    <row r="26" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="G25" s="1"/>
+    </row>
+    <row r="26" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
-    </row>
-    <row r="27" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="G26" s="1"/>
+    </row>
+    <row r="27" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
-    </row>
-    <row r="28" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="G27" s="1"/>
+    </row>
+    <row r="28" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
-    </row>
-    <row r="29" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="G28" s="1"/>
+    </row>
+    <row r="29" spans="4:7" x14ac:dyDescent="0.3">
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1067,11 +1150,14 @@
     <hyperlink ref="F6" r:id="rId3" xr:uid="{72B93DAE-DDC0-4CAC-B2EB-B9DF4045F40A}"/>
     <hyperlink ref="F4" r:id="rId4" xr:uid="{26AFA390-40A5-4FFC-9A26-C0E8B7E0D55B}"/>
     <hyperlink ref="F5" r:id="rId5" xr:uid="{CC656887-3A8F-48AB-AF9F-01D1075CFCC9}"/>
+    <hyperlink ref="G2" r:id="rId6" xr:uid="{57C3F10E-C9EC-442F-B544-CC0FB66C187B}"/>
+    <hyperlink ref="G3" r:id="rId7" xr:uid="{FDC73A8A-2B36-4377-953E-26FB7E348CED}"/>
+    <hyperlink ref="G4" r:id="rId8" xr:uid="{6C39B9F5-6B06-4EFA-9DB2-FA4C3A86BBDD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
   <tableParts count="1">
-    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId10"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>